<commit_message>
created Registration Builder class
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testdata.xlsx
+++ b/src/test/resources/testData/testdata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="84" windowWidth="13332" windowHeight="5544"/>
+    <workbookView xWindow="480" yWindow="84" windowWidth="13332" windowHeight="5544" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="154">
   <si>
     <t>Password_Incorrect</t>
   </si>
@@ -912,7 +912,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="202">
+  <cellXfs count="204">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1497,6 +1497,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1991,7 +1997,7 @@
       <c r="D1" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="202" t="s">
         <v>63</v>
       </c>
       <c r="F1" s="22" t="s">
@@ -2036,8 +2042,8 @@
       <c r="D2" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="131">
-        <v>10101991</v>
+      <c r="E2" s="169" t="s">
+        <v>147</v>
       </c>
       <c r="F2" s="23" t="s">
         <v>75</v>
@@ -2081,7 +2087,7 @@
       <c r="D3" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="131">
+      <c r="E3" s="170">
         <v>10101991</v>
       </c>
       <c r="F3" s="23" t="s">
@@ -2126,8 +2132,8 @@
       <c r="D4" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="131">
-        <v>10101991</v>
+      <c r="E4" s="170" t="s">
+        <v>147</v>
       </c>
       <c r="F4" s="23" t="s">
         <v>75</v>
@@ -2169,8 +2175,8 @@
       <c r="D5" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="131">
-        <v>10101991</v>
+      <c r="E5" s="203" t="s">
+        <v>147</v>
       </c>
       <c r="F5" s="23" t="s">
         <v>75</v>
@@ -2212,8 +2218,8 @@
         <v>82</v>
       </c>
       <c r="D6" s="25"/>
-      <c r="E6" s="133">
-        <v>10101991</v>
+      <c r="E6" s="171" t="s">
+        <v>147</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>75</v>
@@ -2257,8 +2263,8 @@
       <c r="D7" s="27">
         <v>456789456</v>
       </c>
-      <c r="E7" s="134">
-        <v>10101991</v>
+      <c r="E7" s="194" t="s">
+        <v>147</v>
       </c>
       <c r="F7" s="27" t="s">
         <v>75</v>
@@ -2300,8 +2306,8 @@
       <c r="D8" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="E8" s="134">
-        <v>10101991</v>
+      <c r="E8" s="194" t="s">
+        <v>147</v>
       </c>
       <c r="F8" s="27" t="s">
         <v>75</v>
@@ -2343,8 +2349,8 @@
       <c r="D9" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="E9" s="135">
-        <v>10101991</v>
+      <c r="E9" s="195" t="s">
+        <v>147</v>
       </c>
       <c r="F9" s="30" t="s">
         <v>75</v>
@@ -2604,7 +2610,7 @@
       <c r="E15" s="179" t="s">
         <v>147</v>
       </c>
-      <c r="F15" s="33"/>
+      <c r="F15" s="136"/>
       <c r="G15" s="179" t="s">
         <v>143</v>
       </c>
@@ -2647,7 +2653,7 @@
       <c r="E16" s="180" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="137">
         <v>456789123</v>
       </c>
       <c r="G16" s="180" t="s">
@@ -2690,7 +2696,7 @@
       <c r="E17" s="181" t="s">
         <v>147</v>
       </c>
-      <c r="F17" s="36" t="s">
+      <c r="F17" s="138" t="s">
         <v>84</v>
       </c>
       <c r="G17" s="181" t="s">

</xml_diff>